<commit_message>
Benahi baseline perencanaan aset dan master tahun rencana
</commit_message>
<xml_diff>
--- a/modules/apperp/management-aset/resources/laporan/laporan-pengadaan-aset/standar.xlsx
+++ b/modules/apperp/management-aset/resources/laporan/laporan-pengadaan-aset/standar.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Pengadaan aset" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pengadaan aset'!$A$10:$V$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pengadaan aset'!$A$10:$W$10</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="71">
   <si>
     <t>${kop.logo_kiri}</t>
   </si>
@@ -85,6 +85,12 @@
     <t>${filter_tambahan}</t>
   </si>
   <si>
+    <t>Rencana belum diestimasi</t>
+  </si>
+  <si>
+    <t>${jumlah_baris_belum_diestimasi}</t>
+  </si>
+  <si>
     <t>No.</t>
   </si>
   <si>
@@ -101,6 +107,12 @@
   </si>
   <si>
     <t>${baris.tanggal_rencana}</t>
+  </si>
+  <si>
+    <t>Tanggal kebutuhan</t>
+  </si>
+  <si>
+    <t>${baris.tanggal_kebutuhan}</t>
   </si>
   <si>
     <t>Tahun anggaran</t>
@@ -647,34 +659,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:V13"/>
+  <dimension ref="A1:W13"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
     <col min="2" max="2" width="16" customWidth="true" style="0"/>
     <col min="3" max="3" width="13" customWidth="true" style="0"/>
-    <col min="4" max="4" width="10" customWidth="true" style="0"/>
-    <col min="5" max="5" width="16" customWidth="true" style="0"/>
-    <col min="6" max="6" width="26" customWidth="true" style="0"/>
-    <col min="7" max="7" width="28" customWidth="true" style="0"/>
-    <col min="8" max="8" width="9" customWidth="true" style="0"/>
-    <col min="9" max="9" width="10" customWidth="true" style="0"/>
-    <col min="10" max="10" width="18" customWidth="true" style="0"/>
+    <col min="4" max="4" width="13" customWidth="true" style="0"/>
+    <col min="5" max="5" width="10" customWidth="true" style="0"/>
+    <col min="6" max="6" width="16" customWidth="true" style="0"/>
+    <col min="7" max="7" width="26" customWidth="true" style="0"/>
+    <col min="8" max="8" width="28" customWidth="true" style="0"/>
+    <col min="9" max="9" width="9" customWidth="true" style="0"/>
+    <col min="10" max="10" width="10" customWidth="true" style="0"/>
     <col min="11" max="11" width="18" customWidth="true" style="0"/>
-    <col min="12" max="12" width="13" customWidth="true" style="0"/>
-    <col min="13" max="13" width="10" customWidth="true" style="0"/>
+    <col min="12" max="12" width="18" customWidth="true" style="0"/>
+    <col min="13" max="13" width="13" customWidth="true" style="0"/>
     <col min="14" max="14" width="10" customWidth="true" style="0"/>
-    <col min="15" max="15" width="18" customWidth="true" style="0"/>
-    <col min="16" max="16" width="13" customWidth="true" style="0"/>
-    <col min="17" max="17" width="22" customWidth="true" style="0"/>
-    <col min="18" max="18" width="10" customWidth="true" style="0"/>
-    <col min="19" max="19" width="18" customWidth="true" style="0"/>
-    <col min="20" max="20" width="10" customWidth="true" style="0"/>
-    <col min="21" max="21" width="22" customWidth="true" style="0"/>
-    <col min="22" max="22" width="16" customWidth="true" style="0"/>
+    <col min="15" max="15" width="10" customWidth="true" style="0"/>
+    <col min="16" max="16" width="18" customWidth="true" style="0"/>
+    <col min="17" max="17" width="13" customWidth="true" style="0"/>
+    <col min="18" max="18" width="22" customWidth="true" style="0"/>
+    <col min="19" max="19" width="10" customWidth="true" style="0"/>
+    <col min="20" max="20" width="18" customWidth="true" style="0"/>
+    <col min="21" max="21" width="10" customWidth="true" style="0"/>
+    <col min="22" max="22" width="22" customWidth="true" style="0"/>
+    <col min="23" max="23" width="16" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" customHeight="1" ht="22">
+    <row r="1" spans="1:23" customHeight="1" ht="22">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -700,11 +713,12 @@
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
       <c r="U1" s="1"/>
-      <c r="V1" t="s">
+      <c r="V1" s="1"/>
+      <c r="W1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:22" customHeight="1" ht="24">
+    <row r="2" spans="1:23" customHeight="1" ht="24">
       <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
@@ -727,8 +741,9 @@
       <c r="S2" s="1"/>
       <c r="T2" s="1"/>
       <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
     </row>
-    <row r="3" spans="1:22" customHeight="1" ht="22">
+    <row r="3" spans="1:23" customHeight="1" ht="22">
       <c r="A3" s="3"/>
       <c r="B3" s="4" t="s">
         <v>3</v>
@@ -752,14 +767,15 @@
       <c r="S3" s="4"/>
       <c r="T3" s="4"/>
       <c r="U3" s="4"/>
-      <c r="V3" s="3"/>
+      <c r="V3" s="4"/>
+      <c r="W3" s="3"/>
     </row>
-    <row r="5" spans="1:22">
+    <row r="5" spans="1:23">
       <c r="A5" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:22">
+    <row r="6" spans="1:23">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -779,7 +795,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:22">
+    <row r="7" spans="1:23">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -799,7 +815,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:22">
+    <row r="8" spans="1:23">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -813,145 +829,159 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:22" customHeight="1" ht="32">
+    <row r="9" spans="1:23">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" customHeight="1" ht="32">
       <c r="A10" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M10" s="7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="N10" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="O10" s="7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="P10" s="7" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="Q10" s="7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="R10" s="7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="S10" s="7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="T10" s="7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="U10" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="V10" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="V10" s="7" t="s">
+      <c r="W10" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:22">
+    <row r="11" spans="1:23">
       <c r="A11" s="8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="J11" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K11" s="8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L11" s="8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="M11" s="8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="N11" s="8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="O11" s="8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="P11" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="Q11" s="8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="R11" s="8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="S11" s="8" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="T11" s="8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="U11" s="8" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="V11" s="8" t="s">
-        <v>63</v>
+        <v>66</v>
+      </c>
+      <c r="W11" s="8" t="s">
+        <v>67</v>
       </c>
     </row>
-    <row r="13" spans="1:22">
+    <row r="13" spans="1:23">
       <c r="A13" s="9" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -961,10 +991,10 @@
       <c r="G13" s="9"/>
       <c r="H13" s="9"/>
       <c r="I13" s="9"/>
-      <c r="J13" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="K13" s="9"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9" t="s">
+        <v>69</v>
+      </c>
       <c r="L13" s="9"/>
       <c r="M13" s="9"/>
       <c r="N13" s="9"/>
@@ -972,22 +1002,23 @@
       <c r="P13" s="9"/>
       <c r="Q13" s="9"/>
       <c r="R13" s="9"/>
-      <c r="S13" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="T13" s="9"/>
+      <c r="S13" s="9"/>
+      <c r="T13" s="9" t="s">
+        <v>70</v>
+      </c>
       <c r="U13" s="9"/>
       <c r="V13" s="9"/>
+      <c r="W13" s="9"/>
     </row>
   </sheetData>
-  <autoFilter ref="A10:V10"/>
+  <autoFilter ref="A10:W10"/>
   <mergeCells>
     <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:U1"/>
-    <mergeCell ref="B2:U2"/>
-    <mergeCell ref="B3:U3"/>
-    <mergeCell ref="V1:V3"/>
-    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="B1:V1"/>
+    <mergeCell ref="B2:V2"/>
+    <mergeCell ref="B3:V3"/>
+    <mergeCell ref="W1:W3"/>
+    <mergeCell ref="A13:J13"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Benahi perencanaan aset tahunan dan lookup SDK (#362)
* Benahi baseline perencanaan aset dan master tahun rencana

* Tutup celah lookup izin dan lengkapi verifikasi perencanaan

* Pisahkan cursor lookup internal dari request daftar

* Jaga kompatibilitas estimasi dan lengkapi metadata data

* Jadikan migration master mandiri untuk admin.erp

* Hitung estimasi lewat model dengan scope tenant
</commit_message>
<xml_diff>
--- a/modules/apperp/management-aset/resources/laporan/laporan-pengadaan-aset/standar.xlsx
+++ b/modules/apperp/management-aset/resources/laporan/laporan-pengadaan-aset/standar.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Pengadaan aset" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pengadaan aset'!$A$10:$V$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pengadaan aset'!$A$10:$W$10</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="71">
   <si>
     <t>${kop.logo_kiri}</t>
   </si>
@@ -85,6 +85,12 @@
     <t>${filter_tambahan}</t>
   </si>
   <si>
+    <t>Rencana belum diestimasi</t>
+  </si>
+  <si>
+    <t>${jumlah_baris_belum_diestimasi}</t>
+  </si>
+  <si>
     <t>No.</t>
   </si>
   <si>
@@ -101,6 +107,12 @@
   </si>
   <si>
     <t>${baris.tanggal_rencana}</t>
+  </si>
+  <si>
+    <t>Tanggal kebutuhan</t>
+  </si>
+  <si>
+    <t>${baris.tanggal_kebutuhan}</t>
   </si>
   <si>
     <t>Tahun anggaran</t>
@@ -647,34 +659,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:V13"/>
+  <dimension ref="A1:W13"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="true" style="0"/>
     <col min="2" max="2" width="16" customWidth="true" style="0"/>
     <col min="3" max="3" width="13" customWidth="true" style="0"/>
-    <col min="4" max="4" width="10" customWidth="true" style="0"/>
-    <col min="5" max="5" width="16" customWidth="true" style="0"/>
-    <col min="6" max="6" width="26" customWidth="true" style="0"/>
-    <col min="7" max="7" width="28" customWidth="true" style="0"/>
-    <col min="8" max="8" width="9" customWidth="true" style="0"/>
-    <col min="9" max="9" width="10" customWidth="true" style="0"/>
-    <col min="10" max="10" width="18" customWidth="true" style="0"/>
+    <col min="4" max="4" width="13" customWidth="true" style="0"/>
+    <col min="5" max="5" width="10" customWidth="true" style="0"/>
+    <col min="6" max="6" width="16" customWidth="true" style="0"/>
+    <col min="7" max="7" width="26" customWidth="true" style="0"/>
+    <col min="8" max="8" width="28" customWidth="true" style="0"/>
+    <col min="9" max="9" width="9" customWidth="true" style="0"/>
+    <col min="10" max="10" width="10" customWidth="true" style="0"/>
     <col min="11" max="11" width="18" customWidth="true" style="0"/>
-    <col min="12" max="12" width="13" customWidth="true" style="0"/>
-    <col min="13" max="13" width="10" customWidth="true" style="0"/>
+    <col min="12" max="12" width="18" customWidth="true" style="0"/>
+    <col min="13" max="13" width="13" customWidth="true" style="0"/>
     <col min="14" max="14" width="10" customWidth="true" style="0"/>
-    <col min="15" max="15" width="18" customWidth="true" style="0"/>
-    <col min="16" max="16" width="13" customWidth="true" style="0"/>
-    <col min="17" max="17" width="22" customWidth="true" style="0"/>
-    <col min="18" max="18" width="10" customWidth="true" style="0"/>
-    <col min="19" max="19" width="18" customWidth="true" style="0"/>
-    <col min="20" max="20" width="10" customWidth="true" style="0"/>
-    <col min="21" max="21" width="22" customWidth="true" style="0"/>
-    <col min="22" max="22" width="16" customWidth="true" style="0"/>
+    <col min="15" max="15" width="10" customWidth="true" style="0"/>
+    <col min="16" max="16" width="18" customWidth="true" style="0"/>
+    <col min="17" max="17" width="13" customWidth="true" style="0"/>
+    <col min="18" max="18" width="22" customWidth="true" style="0"/>
+    <col min="19" max="19" width="10" customWidth="true" style="0"/>
+    <col min="20" max="20" width="18" customWidth="true" style="0"/>
+    <col min="21" max="21" width="10" customWidth="true" style="0"/>
+    <col min="22" max="22" width="22" customWidth="true" style="0"/>
+    <col min="23" max="23" width="16" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" customHeight="1" ht="22">
+    <row r="1" spans="1:23" customHeight="1" ht="22">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -700,11 +713,12 @@
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
       <c r="U1" s="1"/>
-      <c r="V1" t="s">
+      <c r="V1" s="1"/>
+      <c r="W1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:22" customHeight="1" ht="24">
+    <row r="2" spans="1:23" customHeight="1" ht="24">
       <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
@@ -727,8 +741,9 @@
       <c r="S2" s="1"/>
       <c r="T2" s="1"/>
       <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
     </row>
-    <row r="3" spans="1:22" customHeight="1" ht="22">
+    <row r="3" spans="1:23" customHeight="1" ht="22">
       <c r="A3" s="3"/>
       <c r="B3" s="4" t="s">
         <v>3</v>
@@ -752,14 +767,15 @@
       <c r="S3" s="4"/>
       <c r="T3" s="4"/>
       <c r="U3" s="4"/>
-      <c r="V3" s="3"/>
+      <c r="V3" s="4"/>
+      <c r="W3" s="3"/>
     </row>
-    <row r="5" spans="1:22">
+    <row r="5" spans="1:23">
       <c r="A5" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:22">
+    <row r="6" spans="1:23">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -779,7 +795,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:22">
+    <row r="7" spans="1:23">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -799,7 +815,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:22">
+    <row r="8" spans="1:23">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -813,145 +829,159 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:22" customHeight="1" ht="32">
+    <row r="9" spans="1:23">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" customHeight="1" ht="32">
       <c r="A10" s="7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M10" s="7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="N10" s="7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="O10" s="7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="P10" s="7" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="Q10" s="7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="R10" s="7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="S10" s="7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="T10" s="7" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="U10" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="V10" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="V10" s="7" t="s">
+      <c r="W10" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:22">
+    <row r="11" spans="1:23">
       <c r="A11" s="8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="J11" s="8" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K11" s="8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L11" s="8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="M11" s="8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="N11" s="8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="O11" s="8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="P11" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="Q11" s="8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="R11" s="8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="S11" s="8" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="T11" s="8" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="U11" s="8" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="V11" s="8" t="s">
-        <v>63</v>
+        <v>66</v>
+      </c>
+      <c r="W11" s="8" t="s">
+        <v>67</v>
       </c>
     </row>
-    <row r="13" spans="1:22">
+    <row r="13" spans="1:23">
       <c r="A13" s="9" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -961,10 +991,10 @@
       <c r="G13" s="9"/>
       <c r="H13" s="9"/>
       <c r="I13" s="9"/>
-      <c r="J13" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="K13" s="9"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9" t="s">
+        <v>69</v>
+      </c>
       <c r="L13" s="9"/>
       <c r="M13" s="9"/>
       <c r="N13" s="9"/>
@@ -972,22 +1002,23 @@
       <c r="P13" s="9"/>
       <c r="Q13" s="9"/>
       <c r="R13" s="9"/>
-      <c r="S13" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="T13" s="9"/>
+      <c r="S13" s="9"/>
+      <c r="T13" s="9" t="s">
+        <v>70</v>
+      </c>
       <c r="U13" s="9"/>
       <c r="V13" s="9"/>
+      <c r="W13" s="9"/>
     </row>
   </sheetData>
-  <autoFilter ref="A10:V10"/>
+  <autoFilter ref="A10:W10"/>
   <mergeCells>
     <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:U1"/>
-    <mergeCell ref="B2:U2"/>
-    <mergeCell ref="B3:U3"/>
-    <mergeCell ref="V1:V3"/>
-    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="B1:V1"/>
+    <mergeCell ref="B2:V2"/>
+    <mergeCell ref="B3:V3"/>
+    <mergeCell ref="W1:W3"/>
+    <mergeCell ref="A13:J13"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>